<commit_message>
Updated short notes and provenience info in "pipeline\definitions\indices_manifest.json" and Excel version of the manifest in "data\docs\indices_manifest.xlsx".
</commit_message>
<xml_diff>
--- a/data/docs/indices_manifest.xlsx
+++ b/data/docs/indices_manifest.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Administrative_Indicators" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Folder_Catalog'!$A$1:$H$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Folder_Catalog'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Indices_Summary'!$A$1:$Q$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cell_Vars'!$A$1:$C$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cell_Filters'!$A$1:$E$3</definedName>
@@ -506,7 +506,7 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>- Folder_Catalog: raster folders, descriptions, paths, and TIFF-derived spatial metadata</t>
+          <t>- Folder_Catalog: raster descriptions, source provenance and processing, paths, and TIFF-derived spatial metadata</t>
         </is>
       </c>
     </row>
@@ -580,17 +580,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="57" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -601,35 +602,40 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>provenience</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>folder_path</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>tiff_crs</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>tiff_resolution</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tiff_resolution_unit</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>tiff_pixel_area</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>sample_tiff</t>
         </is>
@@ -643,33 +649,38 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Building age classes / bins</t>
+          <t>Dominant building construction age classes (GHS-AGE).</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-AGE. The generic TIFF curator copies rasters already in Mollweide unchanged and otherwise reprojects them to Mollweide with bilinear resampling. No raster-value transformation is defined; age-class recoding occurs later in index construction.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Age</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>GHS_AGE_1975052020_GLOBE_R2025A_54009_100_V1_0.tif</t>
         </is>
@@ -683,33 +694,38 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Height raster(s)</t>
+          <t>Gridded building height (GHS-BUILT-H).</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-BUILT-H, epoch 2018; local inventory filenames identify 100 m Mollweide (54009) tiles. The generic curator therefore copies these already-Mollweide rasters unchanged; no value transformation is defined.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Height</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>GHS_BUILT_H_AGBH_E2018_GLOBE_R2023A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -723,33 +739,38 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Population raster(s)</t>
+          <t>Gridded population count (GHS-POP).</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-POP, epoch 2010; local inventory filenames identify 100 m Mollweide (54009) tiles. The generic curator therefore copies these already-Mollweide rasters unchanged; no value transformation is defined.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Population</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>GHS_POP_E2010_GLOBE_R2023A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -763,33 +784,38 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Residential built-up surface</t>
+          <t>Residential built-up surface.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-BUILT-S. The generic TIFF curator copies inputs already in Mollweide and otherwise reprojects to Mollweide with bilinear resampling; it does not transform pixel values. The repository code does not document how the residential component was separated from the downloaded product.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Surface</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>GHS_BUILT_S_E2010_GLOBE_R2023A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -803,33 +829,38 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Non-residential built-up surface</t>
+          <t>Non-residential built-up surface.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-BUILT-S. The generic TIFF curator copies inputs already in Mollweide and otherwise reprojects to Mollweide with bilinear resampling; it does not transform pixel values. The repository code does not document how the non-residential component was separated from the downloaded product.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Surface_NRES</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>GHS_BUILT_S_NRES_E2010_GLOBE_R2023A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -843,33 +874,38 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Residential volume raster(s)</t>
+          <t>Residential built-up volume.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-BUILT-V (2010; source download notes specify WGS84, 3-arc-second tiles). The generic TIFF curator reprojects non-Mollweide inputs to Mollweide with bilinear resampling, changing the grid but not applying a thematic value transform. The residential/non-residential derivation is not documented in preprocessing code.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Volume</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>GHS_BUILT_V_E2010_GLOBE_R2023A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -883,33 +919,38 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Non-residential volume raster(s)</t>
+          <t>Non-residential built-up volume.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-BUILT-V (2010; source download notes specify WGS84, 3-arc-second tiles). The generic TIFF curator reprojects non-Mollweide inputs to Mollweide with bilinear resampling, changing the grid but not applying a thematic value transform. The non-residential derivation is not documented in preprocessing code.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Volume_NRES</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>GHS_BUILT_V_NRES_E2010_GLOBE_R2023A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -923,33 +964,38 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Night-time lights intensity raster(s)</t>
+          <t>Annual VIIRS night-time light radiance.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>Source: NOAA/EOG VIIRS annual VNL product (2012). curate_raw_tiffs.py applies ln(x + 2) to band 1 and targets a 1,000 m Mollweide grid; non-Mollweide inputs are bilinearly resampled during reprojection. This is a substantive pixel-value transform plus spatial resampling.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\NTL</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>PROJCS["unknown",GEOGCS["unknown",DATUM["WGS_1984",SPHEROID["WGS 84",6378137,298.257223563,AUTHORITY["EPSG","7030"]],AUTHORITY["EPSG","6326"]],PRIMEM["Greenwich",0],UNIT["Degree",0.0174532925199433]],PROJECTION["Mollweide"],PARAMETER["central_meridian",0],PARAMETER["false_easting",0],PARAMETER["false_northing",0],UNIT["metre",1,AUTHORITY["EPSG","9001"]],AXIS["Easting",EAST],AXIS["Northing",NORTH]]</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>257.276 x 257.276</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>66190.96703456134</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>VNL_v21_npp_201204-201212_global_vcmcfg_c202205302300.median_masked.dat.tif</t>
         </is>
@@ -963,33 +1009,38 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PM2.5 annual/overall average raster(s)</t>
+          <t>Mean monthly PM2.5 concentration for 2010-2012.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>Source: SatPM monthly gridded PM2.5. curate_pm_2_5.py masks values below -100, computes the mean of available monthly values for 2010-2012, then reprojects to Mollweide at 1,000 m with rioxarray using its default nearest-neighbor resampling. This is a derived temporal summary plus spatial resampling.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\PM_2_5_average</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>1000 x 1000</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>1000000</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>pm25_average_2010_2012_mollweide.tif</t>
         </is>
@@ -1003,33 +1054,38 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PM2.5 heating-season delta raster(s)</t>
+          <t>Heating-season PM2.5 difference: January-February mean minus March-December mean, averaged over 2010-2012.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>Source: SatPM monthly gridded PM2.5. curate_pm_2_5.py masks values below -100, calculates each year's Jan-Feb mean minus the remaining-month mean, averages the yearly differences for 2010-2012, then reprojects to Mollweide at 1,000 m using nearest-neighbor resampling. This is a derived seasonal contrast plus spatial resampling.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\PM_2_5_delta</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>1000 x 1000</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>1000000</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>pm25_delta_JanFeb_minus_rest_2010_2012_mollweide.tif</t>
         </is>
@@ -1043,33 +1099,38 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Black carbon average raster(s)</t>
+          <t>Mean monthly residential black-carbon emissions for 2010-2012.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>Source: CAMS-GLOB-ANT monthly residential BC flux (kg/m2/s). curate_oc_bc.py handles fill values, converts flux to monthly mass using days per month, averages valid months across 2010-2012, then reprojects to Mollweide at 10,000 m. This is a derived temporal/unit transformation plus spatial resampling.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\BC_average</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>10000 x 10000</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>100000000</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>bc_average_2010_2012_mollweide.tif</t>
         </is>
@@ -1083,33 +1144,38 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Black carbon heating-season delta raster(s)</t>
+          <t>Residential black-carbon emissions difference: January-February mean minus March-December mean, averaged over 2010-2012.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>Source: CAMS-GLOB-ANT monthly residential BC flux (kg/m2/s). curate_oc_bc.py handles fill values, converts to monthly mass, computes each year's Jan-Feb minus remaining-month mean, averages yearly differences for 2010-2012, then reprojects to Mollweide at 10,000 m.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\BC_delta</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>10000 x 10000</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>100000000</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>bc_delta_JanFeb_minus_rest_2010_2012_mollweide.tif</t>
         </is>
@@ -1123,33 +1189,38 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Organic carbon average raster(s)</t>
+          <t>Mean monthly residential organic-carbon emissions for 2010-2012.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t>Source: CAMS-GLOB-ANT monthly residential OC flux (kg/m2/s). curate_oc_bc.py handles fill values, converts flux to monthly mass using days per month, averages valid months across 2010-2012, then reprojects to Mollweide at 10,000 m. This is a derived temporal/unit transformation plus spatial resampling.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\OC_average</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>10000 x 10000</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>100000000</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>oc_average_2010_2012_mollweide.tif</t>
         </is>
@@ -1163,33 +1234,38 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Organic carbon heating-season delta raster(s)</t>
+          <t>Residential organic-carbon emissions difference: January-February mean minus March-December mean, averaged over 2010-2012.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
+          <t>Source: CAMS-GLOB-ANT monthly residential OC flux (kg/m2/s). curate_oc_bc.py handles fill values, converts to monthly mass, computes each year's Jan-Feb minus remaining-month mean, averages yearly differences for 2010-2012, then reprojects to Mollweide at 10,000 m.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\OC_delta</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>10000 x 10000</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>100000000</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>oc_delta_JanFeb_minus_rest_2010_2012_mollweide.tif</t>
         </is>
@@ -1203,33 +1279,38 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Heating degree days</t>
+          <t>Mean annual count of days with daily mean ERA5-Land skin temperature below 18 degrees C (2010-2012).</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
+          <t>Source: ECMWF ERA5-Land DAILY_AGGR skin_temperature; computed in the included Google Colab/GEE notebook, not in a locally runnable pipeline step. It converts K to degrees C, counts qualifying days per year, then averages the annual maps for 2010-2012. curate_raw_tiffs.py force-reprojects the exported native-grid GeoTIFF to Mollweide with bilinear resampling.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\ERA5-Land_HDD</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>PROJCS["unknown",GEOGCS["unknown",DATUM["WGS_1984",SPHEROID["WGS 84",6378137,298.257223563,AUTHORITY["EPSG","7030"]],AUTHORITY["EPSG","6326"]],PRIMEM["Greenwich",0],UNIT["Degree",0.0174532925199433]],PROJECTION["Mollweide"],PARAMETER["central_meridian",0],PARAMETER["false_easting",0],PARAMETER["false_northing",0],UNIT["metre",1,AUTHORITY["EPSG","9001"]],AXIS["Easting",EAST],AXIS["Northing",NORTH]]</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>8832.36 x 8832.36</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>78010538.90945257</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>PT_hdd_18_ERA5L_skinT_dailyMean_2010_2012_nativegrid.tif</t>
         </is>
@@ -1243,33 +1324,38 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Cooling degree days</t>
+          <t>Mean annual count of days with daily mean ERA5-Land skin temperature above 25 degrees C (2010-2012).</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
+          <t>Source: ECMWF ERA5-Land DAILY_AGGR skin_temperature; computed in the included Google Colab/GEE notebook, not in a locally runnable pipeline step. It converts K to degrees C, counts qualifying days per year, then averages the annual maps for 2010-2012. curate_raw_tiffs.py force-reprojects the exported native-grid GeoTIFF to Mollweide with bilinear resampling.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\ERA5-Land_CDD</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>PROJCS["unknown",GEOGCS["unknown",DATUM["WGS_1984",SPHEROID["WGS 84",6378137,298.257223563,AUTHORITY["EPSG","7030"]],AUTHORITY["EPSG","6326"]],PRIMEM["Greenwich",0],UNIT["Degree",0.0174532925199433]],PROJECTION["Mollweide"],PARAMETER["central_meridian",0],PARAMETER["false_easting",0],PARAMETER["false_northing",0],UNIT["metre",1,AUTHORITY["EPSG","9001"]],AXIS["Easting",EAST],AXIS["Northing",NORTH]]</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>8832.36 x 8832.36</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>78010538.90945257</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>PT_cdd_25_ERA5L_skinT_dailyMean_2010_2012_nativegrid.tif</t>
         </is>
@@ -1283,33 +1369,38 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>6th–10th hottest days mean temperature</t>
+          <t>Mean across 2010-2012 of each year's mean daily temperature among the 6th-10th hottest days.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>Source: ECMWF ERA5-Land DAILY_AGGR skin_temperature; computed in the included Google Colab/GEE notebook, not in a locally runnable pipeline step. It converts K to degrees C, selects the 6th-10th hottest daily values per year and pixel, averages those five, then averages yearly maps. The exported native-grid TIFF is force-reprojected to Mollweide with bilinear resampling by curate_raw_tiffs.py.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\ERA5-Land_extreme_heat</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>PROJCS["unknown",GEOGCS["unknown",DATUM["WGS_1984",SPHEROID["WGS 84",6378137,298.257223563,AUTHORITY["EPSG","7030"]],AUTHORITY["EPSG","6326"]],PRIMEM["Greenwich",0],UNIT["Degree",0.0174532925199433]],PROJECTION["Mollweide"],PARAMETER["central_meridian",0],PARAMETER["false_easting",0],PARAMETER["false_northing",0],UNIT["metre",1,AUTHORITY["EPSG","9001"]],AXIS["Easting",EAST],AXIS["Northing",NORTH]]</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>8832.36 x 8832.36</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>78010538.90945257</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>PT_extreme_heat_ERA5L_skinT_dailyMean_2010_2012_nativegrid.tif</t>
         </is>
@@ -1323,33 +1414,38 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>6th–10th coldest days mean temperature</t>
+          <t>Mean across 2010-2012 of each year's mean daily temperature among the 6th-10th coldest days.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
+          <t>Source: ECMWF ERA5-Land DAILY_AGGR skin_temperature; computed in the included Google Colab/GEE notebook, not in a locally runnable pipeline step. It converts K to degrees C, selects the 6th-10th coldest daily values per year and pixel, averages those five, then averages yearly maps. The exported native-grid TIFF is force-reprojected to Mollweide with bilinear resampling by curate_raw_tiffs.py.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\ERA5-Land_extreme_cold</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>PROJCS["unknown",GEOGCS["unknown",DATUM["WGS_1984",SPHEROID["WGS 84",6378137,298.257223563,AUTHORITY["EPSG","7030"]],AUTHORITY["EPSG","6326"]],PRIMEM["Greenwich",0],UNIT["Degree",0.0174532925199433]],PROJECTION["Mollweide"],PARAMETER["central_meridian",0],PARAMETER["false_easting",0],PARAMETER["false_northing",0],UNIT["metre",1,AUTHORITY["EPSG","9001"]],AXIS["Easting",EAST],AXIS["Northing",NORTH]]</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>8832.36 x 8832.36</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>78010538.90945257</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>PT_extreme_cold_ERA5L_skinT_dailyMean_2010_2012_nativegrid.tif</t>
         </is>
@@ -1363,33 +1459,38 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Greenness vegetation proxy (if used later)</t>
+          <t>Built-up greenness proxy (planned/optional input).</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
+          <t>Source: EMC built greenness product (local inventory identifies a 2022 100 m Mollweide product). If curated through curate_raw_tiffs.py, already-Mollweide TIFFs are copied and other CRSs are reprojected to Mollweide with bilinear resampling; no value transform is defined. Not currently selected as a pipeline input.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\Greenness</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>100 x 100</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EMC_BUILT_GREENNESS_E2022_GLOBE_R2025A_54009_100_V1_0_R4_C18.tif</t>
         </is>
@@ -1403,40 +1504,45 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Settlement model degree of urbanization (if used later)</t>
+          <t>Settlement Model degree-of-urbanisation classes (planned/optional input).</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
+          <t>Source: JRC GHSL GHS-SMOD (local inventory identifies a 2010 1 km Mollweide product). If curated through curate_raw_tiffs.py, already-Mollweide TIFFs are copied and other CRSs are reprojected to Mollweide with bilinear resampling; no value transform is defined. Not currently selected as a pipeline input.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
           <t>E:\OneDrive\Studia\Studia magisterskie\Masterarbeit 2 - Sozialwissenschaften\data\Sat_data_curated\SMOD</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>ESRI:54009</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>1000 x 1000</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>CRS units; meters for Mollweide</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>1000000</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>GHS_SMOD_E2010_GLOBE_R2023A_54009_1000_V2_0_R4_C18.tif</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H21"/>
+  <autoFilter ref="A1:I21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>